<commit_message>
feat: improve web app, single-card merge, timemark editor, and update docs
</commit_message>
<xml_diff>
--- a/logs/edit_stages.xlsx
+++ b/logs/edit_stages.xlsx
@@ -427,14 +427,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -473,22 +473,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BTP BD\PTDS\COS\0.jpg</t>
+          <t>BTP JAK\SERAT OPTIK\JPL 01 BOO\0.jpg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>stage_1c_guide_original</t>
+          <t>stage_0_override</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PTDS</t>
+          <t>SERAT OPTIK</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>COS</t>
+          <t>JPL 01 BOO</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -498,14 +498,14 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-02 01:10:20</t>
+          <t>2026-09-24 07:36:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BTP BD\PTDS\COS\100.jpg</t>
+          <t>BTP JAK\SERAT OPTIK\JPL 01 BOO\100.jpg</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,12 +515,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PTDS</t>
+          <t>SERAT OPTIK</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>COS</t>
+          <t>JPL 01 BOO</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -530,14 +530,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-02 01:10:20</t>
+          <t>2026-09-24 07:36:04</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BTP BD\PTDS\COS\50.jpg</t>
+          <t>BTP JAK\SERAT OPTIK\JPL 01 BOO\100.original_backup.jpg</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -547,22 +547,54 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PTDS</t>
+          <t>SERAT OPTIK</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>COS</t>
+          <t>JPL 01 BOO</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>100.original_backup.jpg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:36:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BTP JAK\SERAT OPTIK\JPL 01 BOO\50.jpg</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>stage_0_override</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SERAT OPTIK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>JPL 01 BOO</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>50.jpg</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-09-02 01:10:20</t>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:36:04</t>
         </is>
       </c>
     </row>

</xml_diff>